<commit_message>
Add Microsoft downloads; refresh Alphabet to Q2 2026
</commit_message>
<xml_diff>
--- a/assets/files/alphabet-financial-model.xlsx
+++ b/assets/files/alphabet-financial-model.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Comps" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Income Statement'!$A$1:$G$32</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Balance Sheet'!$A$1:$G$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Income Statement'!$A$1:$H$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Balance Sheet'!$A$1:$H$45</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Cash Flow Statement'!$A$1:$I$36</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Key Metrics'!$A$1:$L$31</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Revenue Breakdown'!$A$1:$F$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'SOTP'!$A$1:$F$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Revenue Breakdown'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'SOTP'!$A$1:$F$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Model Inputs'!$A$1:$E$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Peer Comps'!$A$1:$D$19</definedName>
   </definedNames>
@@ -365,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -467,6 +467,47 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -727,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="61" min="1" max="1"/>
@@ -771,6 +812,11 @@
       <c r="G2" s="4" t="n">
         <v>2025</v>
       </c>
+      <c r="H2" s="75" t="inlineStr">
+        <is>
+          <t>Q2 2026A</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="61">
       <c r="A3" s="5" t="n"/>
@@ -818,6 +864,9 @@
       <c r="G5" s="10" t="n">
         <v>402836</v>
       </c>
+      <c r="H5" s="10" t="n">
+        <v>119796</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="61">
       <c r="A6" s="5" t="n"/>
@@ -868,6 +917,9 @@
       <c r="G8" s="15" t="n">
         <v>162535</v>
       </c>
+      <c r="H8" s="76" t="n">
+        <v>45943</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
       <c r="A9" s="9" t="inlineStr">
@@ -897,6 +949,10 @@
       </c>
       <c r="G9" s="10">
         <f>G5-G8</f>
+        <v/>
+      </c>
+      <c r="H9" s="10">
+        <f>H5-H8</f>
         <v/>
       </c>
     </row>
@@ -946,6 +1002,9 @@
       <c r="G12" s="15" t="n">
         <v>61087</v>
       </c>
+      <c r="H12" s="76" t="n">
+        <v>18219</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="12" t="inlineStr">
@@ -971,6 +1030,9 @@
       <c r="G13" s="18" t="n">
         <v>50175</v>
       </c>
+      <c r="H13" s="77" t="n">
+        <v>14864</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="61">
       <c r="A14" s="9" t="inlineStr">
@@ -1000,6 +1062,10 @@
       </c>
       <c r="G14" s="10">
         <f>G12+G13</f>
+        <v/>
+      </c>
+      <c r="H14" s="10">
+        <f>H12+H13</f>
         <v/>
       </c>
     </row>
@@ -1042,6 +1108,10 @@
         <f>G9-G14</f>
         <v/>
       </c>
+      <c r="H16" s="10">
+        <f>H9-H14</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="61">
       <c r="A17" s="5" t="n"/>
@@ -1089,6 +1159,9 @@
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
+      <c r="H19" s="76" t="n">
+        <v>1430</v>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="61">
       <c r="A20" s="12" t="inlineStr">
@@ -1114,6 +1187,9 @@
       <c r="G20" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="H20" s="77" t="n">
+        <v>-1278</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="14" t="inlineStr">
@@ -1139,6 +1215,9 @@
       <c r="G21" s="15" t="n">
         <v>29787</v>
       </c>
+      <c r="H21" s="76" t="n">
+        <v>97831</v>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="61">
       <c r="A22" s="12" t="inlineStr">
@@ -1168,6 +1247,10 @@
       </c>
       <c r="G22" s="13">
         <f>G19+G20+G21</f>
+        <v/>
+      </c>
+      <c r="H22" s="78">
+        <f>H19+H20+H21</f>
         <v/>
       </c>
     </row>
@@ -1210,6 +1293,10 @@
         <f>G16+G22</f>
         <v/>
       </c>
+      <c r="H24" s="78">
+        <f>H16+H22</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="5" t="n"/>
@@ -1244,6 +1331,9 @@
       <c r="G26" s="18" t="n">
         <v>26656</v>
       </c>
+      <c r="H26" s="77" t="n">
+        <v>26560</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="5" t="n"/>
@@ -1284,6 +1374,10 @@
         <f>G24-G26</f>
         <v/>
       </c>
+      <c r="H28" s="10">
+        <f>H24-H26</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="5" t="n"/>
@@ -1337,6 +1431,10 @@
         <f>G28/G32</f>
         <v/>
       </c>
+      <c r="H31" s="79">
+        <f>H28/H32</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="61">
       <c r="A32" s="12" t="inlineStr">
@@ -1362,10 +1460,14 @@
       <c r="G32" s="18" t="n">
         <v>12230</v>
       </c>
+      <c r="H32" s="77" t="n">
+        <v>12309</v>
+      </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -1376,7 +1478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="61" min="1" max="1"/>
@@ -1420,6 +1522,11 @@
       <c r="G2" s="4" t="n">
         <v>2025</v>
       </c>
+      <c r="H2" s="75" t="inlineStr">
+        <is>
+          <t>30-Jun-2026A</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="61">
       <c r="A3" s="5" t="n"/>
@@ -1480,6 +1587,9 @@
       <c r="G6" s="15" t="n">
         <v>30708</v>
       </c>
+      <c r="H6" s="76" t="n">
+        <v>55911</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="12" t="inlineStr">
@@ -1505,6 +1615,9 @@
       <c r="G7" s="18" t="n">
         <v>96135</v>
       </c>
+      <c r="H7" s="77" t="n">
+        <v>186563</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="61">
       <c r="A8" s="14" t="inlineStr">
@@ -1530,6 +1643,9 @@
       <c r="G8" s="15" t="n">
         <v>62886</v>
       </c>
+      <c r="H8" s="76" t="n">
+        <v>69175</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
       <c r="A9" s="12" t="inlineStr">
@@ -1555,6 +1671,9 @@
       <c r="G9" s="18" t="n">
         <v>16309</v>
       </c>
+      <c r="H9" s="77" t="n">
+        <v>31875</v>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="61">
       <c r="A10" s="9" t="inlineStr">
@@ -1584,6 +1703,10 @@
       </c>
       <c r="G10" s="10">
         <f>SUM(G6:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="10">
+        <f>SUM(H6:H9)</f>
         <v/>
       </c>
     </row>
@@ -1633,6 +1756,9 @@
       <c r="G13" s="15" t="n">
         <v>246597</v>
       </c>
+      <c r="H13" s="76" t="n">
+        <v>321212</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="61">
       <c r="A14" s="12" t="inlineStr">
@@ -1658,6 +1784,9 @@
       <c r="G14" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="H14" s="77" t="n">
+        <v>9105</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="61">
       <c r="A15" s="14" t="inlineStr">
@@ -1683,6 +1812,9 @@
       <c r="G15" s="15" t="n">
         <v>33380</v>
       </c>
+      <c r="H15" s="76" t="n">
+        <v>57828</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="61">
       <c r="A16" s="12" t="inlineStr">
@@ -1708,6 +1840,9 @@
       <c r="G16" s="18" t="n">
         <v>68687</v>
       </c>
+      <c r="H16" s="77" t="n">
+        <v>131461</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="61">
       <c r="A17" s="14" t="inlineStr">
@@ -1733,6 +1868,9 @@
       <c r="G17" s="15" t="n">
         <v>40579</v>
       </c>
+      <c r="H17" s="76" t="n">
+        <v>58853</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="61">
       <c r="A18" s="9" t="inlineStr">
@@ -1762,6 +1900,10 @@
       </c>
       <c r="G18" s="10">
         <f>SUM(G13:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="10">
+        <f>SUM(H13:H17)</f>
         <v/>
       </c>
     </row>
@@ -1804,6 +1946,10 @@
         <f>G10+G18</f>
         <v/>
       </c>
+      <c r="H20" s="10">
+        <f>H10+H18</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="5" t="n"/>
@@ -1864,6 +2010,9 @@
       <c r="G24" s="15" t="n">
         <v>12200</v>
       </c>
+      <c r="H24" s="76" t="n">
+        <v>20258</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="12" t="inlineStr">
@@ -1889,6 +2038,9 @@
       <c r="G25" s="18" t="n">
         <v>83967</v>
       </c>
+      <c r="H25" s="77" t="n">
+        <v>88100</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="14" t="inlineStr">
@@ -1914,6 +2066,9 @@
       <c r="G26" s="15" t="n">
         <v>6578</v>
       </c>
+      <c r="H26" s="76" t="n">
+        <v>7154</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="12" t="inlineStr">
@@ -1939,6 +2094,9 @@
       <c r="G27" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="H27" s="77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="61">
       <c r="A28" s="14" t="inlineStr">
@@ -1964,6 +2122,9 @@
       <c r="G28" s="15" t="n">
         <v>0</v>
       </c>
+      <c r="H28" s="76" t="n">
+        <v>10599</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="9" t="inlineStr">
@@ -1993,6 +2154,10 @@
       </c>
       <c r="G29" s="10">
         <f>SUM(G24:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="10">
+        <f>SUM(H24:H28)</f>
         <v/>
       </c>
     </row>
@@ -2042,6 +2207,9 @@
       <c r="G32" s="15" t="n">
         <v>46547</v>
       </c>
+      <c r="H32" s="76" t="n">
+        <v>98165</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="61">
       <c r="A33" s="12" t="inlineStr">
@@ -2067,6 +2235,9 @@
       <c r="G33" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="H33" s="77" t="n">
+        <v>22819</v>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="61">
       <c r="A34" s="14" t="inlineStr">
@@ -2092,6 +2263,9 @@
       <c r="G34" s="15" t="n">
         <v>30724</v>
       </c>
+      <c r="H34" s="76" t="n">
+        <v>34408</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="61">
       <c r="A35" s="9" t="inlineStr">
@@ -2121,6 +2295,10 @@
       </c>
       <c r="G35" s="10">
         <f>G32+G33+G34</f>
+        <v/>
+      </c>
+      <c r="H35" s="10">
+        <f>H32+H33+H34</f>
         <v/>
       </c>
     </row>
@@ -2163,6 +2341,10 @@
         <f>G29+G35</f>
         <v/>
       </c>
+      <c r="H37" s="10">
+        <f>H29+H35</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="61">
       <c r="A38" s="5" t="n"/>
@@ -2210,6 +2392,9 @@
       <c r="G40" s="15" t="n">
         <v>93126</v>
       </c>
+      <c r="H40" s="76" t="n">
+        <v>149394</v>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="61">
       <c r="A41" s="12" t="inlineStr">
@@ -2235,6 +2420,9 @@
       <c r="G41" s="18" t="n">
         <v>324055</v>
       </c>
+      <c r="H41" s="77" t="n">
+        <v>493371</v>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="61">
       <c r="A42" s="14" t="inlineStr">
@@ -2260,6 +2448,9 @@
       <c r="G42" s="15" t="n">
         <v>-1916</v>
       </c>
+      <c r="H42" s="76" t="n">
+        <v>-2285</v>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="61">
       <c r="A43" s="9" t="inlineStr">
@@ -2289,6 +2480,10 @@
       </c>
       <c r="G43" s="10">
         <f>SUM(G40:G42)</f>
+        <v/>
+      </c>
+      <c r="H43" s="10">
+        <f>SUM(H40:H42)</f>
         <v/>
       </c>
     </row>
@@ -2331,10 +2526,15 @@
         <f>G37+G43</f>
         <v/>
       </c>
+      <c r="H45" s="10">
+        <f>H37+H43</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -2391,6 +2591,11 @@
       <c r="G2" s="4" t="n">
         <v>2025</v>
       </c>
+      <c r="H2" s="75" t="inlineStr">
+        <is>
+          <t>H1 2026A</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="61">
       <c r="A3" s="5" t="n"/>
@@ -2438,6 +2643,9 @@
       <c r="G5" s="10" t="n">
         <v>132170</v>
       </c>
+      <c r="H5" s="10" t="n">
+        <v>174771</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="61">
       <c r="A6" s="12" t="inlineStr">
@@ -2463,6 +2671,9 @@
       <c r="G6" s="18" t="n">
         <v>21136</v>
       </c>
+      <c r="H6" s="77" t="n">
+        <v>13586</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="14" t="inlineStr">
@@ -2488,6 +2699,9 @@
       <c r="G7" s="15" t="n">
         <v>24953</v>
       </c>
+      <c r="H7" s="76" t="n">
+        <v>14708</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="61">
       <c r="A8" s="12" t="inlineStr">
@@ -2512,6 +2726,9 @@
       </c>
       <c r="G8" s="18" t="n">
         <v>8348</v>
+      </c>
+      <c r="H8" s="77" t="n">
+        <v>27538</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
@@ -2552,6 +2769,9 @@
       <c r="G10" s="15" t="n">
         <v>-8779</v>
       </c>
+      <c r="H10" s="76" t="n">
+        <v>-6904</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="61">
       <c r="A11" s="12" t="inlineStr">
@@ -2577,6 +2797,9 @@
       <c r="G11" s="18" t="n">
         <v>907</v>
       </c>
+      <c r="H11" s="77" t="n">
+        <v>2090</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="61">
       <c r="A12" s="14" t="inlineStr">
@@ -2602,6 +2825,9 @@
       <c r="G12" s="15" t="n">
         <v>-14022</v>
       </c>
+      <c r="H12" s="76" t="n">
+        <v>-140930</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="9" t="inlineStr">
@@ -2631,6 +2857,10 @@
       </c>
       <c r="G13" s="10">
         <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="10">
+        <f>SUM(H5:H12)</f>
         <v/>
       </c>
     </row>
@@ -2680,6 +2910,9 @@
       <c r="G16" s="15" t="n">
         <v>-91447</v>
       </c>
+      <c r="H16" s="76" t="n">
+        <v>-80598</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="61">
       <c r="A17" s="12" t="inlineStr">
@@ -2705,7 +2938,9 @@
       <c r="G17" s="18" t="n">
         <v>-109489</v>
       </c>
-      <c r="H17" s="23" t="n"/>
+      <c r="H17" s="77" t="n">
+        <v>-98531</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="61">
       <c r="A18" s="14" t="inlineStr">
@@ -2731,6 +2966,9 @@
       <c r="G18" s="15" t="n">
         <v>84607</v>
       </c>
+      <c r="H18" s="76" t="n">
+        <v>68363</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="61">
       <c r="A19" s="12" t="inlineStr">
@@ -2756,6 +2994,9 @@
       <c r="G19" s="18" t="n">
         <v>-1592</v>
       </c>
+      <c r="H19" s="77" t="n">
+        <v>-33697</v>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="61">
       <c r="A20" s="14" t="inlineStr">
@@ -2781,6 +3022,9 @@
       <c r="G20" s="15" t="n">
         <v>-2370</v>
       </c>
+      <c r="H20" s="76" t="n">
+        <v>-1359</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="9" t="inlineStr">
@@ -2806,7 +3050,9 @@
       <c r="G21" s="10" t="n">
         <v>-120291</v>
       </c>
-      <c r="H21" s="23" t="n"/>
+      <c r="H21" s="10" t="n">
+        <v>-145822</v>
+      </c>
       <c r="I21" s="23" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="61">
@@ -2855,6 +3101,9 @@
       <c r="G24" s="15" t="n">
         <v>64564</v>
       </c>
+      <c r="H24" s="76" t="n">
+        <v>56226</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="12" t="inlineStr">
@@ -2880,6 +3129,9 @@
       <c r="G25" s="18" t="n">
         <v>-32427</v>
       </c>
+      <c r="H25" s="77" t="n">
+        <v>-5253</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="14" t="inlineStr">
@@ -2905,6 +3157,9 @@
       <c r="G26" s="15" t="n">
         <v>-45709</v>
       </c>
+      <c r="H26" s="76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="12" t="inlineStr">
@@ -2930,7 +3185,9 @@
       <c r="G27" s="18" t="n">
         <v>-10049</v>
       </c>
-      <c r="H27" s="23" t="n"/>
+      <c r="H27" s="77" t="n">
+        <v>-5231</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="61">
       <c r="A28" s="14" t="inlineStr">
@@ -2956,6 +3213,9 @@
       <c r="G28" s="15" t="n">
         <v>-13767</v>
       </c>
+      <c r="H28" s="76" t="n">
+        <v>40578</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="9" t="inlineStr">
@@ -2985,6 +3245,10 @@
       </c>
       <c r="G29" s="10">
         <f>SUM(G24:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="10">
+        <f>SUM(H24:H28)</f>
         <v/>
       </c>
     </row>
@@ -3027,7 +3291,10 @@
         <f>G13+G21+G29</f>
         <v/>
       </c>
-      <c r="H31" s="23" t="n"/>
+      <c r="H31" s="10">
+        <f>H13+H21+H29</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="61">
       <c r="A32" s="12" t="inlineStr">
@@ -3053,6 +3320,9 @@
       <c r="G32" s="18" t="n">
         <v>23466</v>
       </c>
+      <c r="H32" s="77" t="n">
+        <v>30708</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="61">
       <c r="A33" s="14" t="inlineStr">
@@ -3077,6 +3347,9 @@
       </c>
       <c r="G33" s="15" t="n">
         <v>30708</v>
+      </c>
+      <c r="H33" s="76" t="n">
+        <v>55911</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="61">
@@ -3125,10 +3398,14 @@
       <c r="G36" s="10" t="n">
         <v>73266</v>
       </c>
+      <c r="H36" s="10" t="n">
+        <v>4261</v>
+      </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -3727,8 +4004,9 @@
   <mergeCells count="1">
     <mergeCell ref="I5:L5"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -3739,7 +4017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="37.33203125" customWidth="1" style="61" min="1" max="1"/>
@@ -3779,6 +4057,11 @@
       <c r="F2" s="4" t="n">
         <v>2024</v>
       </c>
+      <c r="G2" s="75" t="inlineStr">
+        <is>
+          <t>Q2 2026A</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="61">
       <c r="A3" s="5" t="n"/>
@@ -3821,6 +4104,9 @@
       <c r="F5" s="30" t="n">
         <v>197868</v>
       </c>
+      <c r="G5" s="80" t="n">
+        <v>63271</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="61">
       <c r="A6" s="12" t="inlineStr">
@@ -3843,6 +4129,9 @@
       <c r="F6" s="28" t="n">
         <v>35309</v>
       </c>
+      <c r="G6" s="81" t="n">
+        <v>11055</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="14" t="inlineStr">
@@ -3865,6 +4154,9 @@
       <c r="F7" s="30" t="n">
         <v>31010</v>
       </c>
+      <c r="G7" s="80" t="n">
+        <v>7303</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="61">
       <c r="A8" s="12" t="inlineStr">
@@ -3887,6 +4179,9 @@
       <c r="F8" s="28" t="n">
         <v>40710</v>
       </c>
+      <c r="G8" s="81" t="n">
+        <v>12911</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
       <c r="A9" s="9" t="inlineStr">
@@ -3912,6 +4207,10 @@
       </c>
       <c r="F9" s="31">
         <f>SUM(F5:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="31">
+        <f>SUM(G5:G8)</f>
         <v/>
       </c>
     </row>
@@ -3956,6 +4255,9 @@
       <c r="F12" s="30" t="n">
         <v>41794</v>
       </c>
+      <c r="G12" s="80" t="n">
+        <v>24768</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="5" t="n"/>
@@ -3998,6 +4300,9 @@
       <c r="F15" s="30" t="n">
         <v>1907</v>
       </c>
+      <c r="G15" s="80" t="n">
+        <v>382</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="61">
       <c r="A16" s="5" t="n"/>
@@ -4040,6 +4345,9 @@
       <c r="F18" s="34" t="n">
         <v>420</v>
       </c>
+      <c r="G18" s="82" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="61">
       <c r="A19" s="5" t="n"/>
@@ -4071,6 +4379,10 @@
       <c r="F20" s="29" t="n">
         <v>350018</v>
       </c>
+      <c r="G20" s="29">
+        <f>G9+G12+G15+G18</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="5" t="n"/>
@@ -4113,6 +4425,9 @@
       <c r="F23" s="29" t="n">
         <v>117372</v>
       </c>
+      <c r="G23" s="29" t="n">
+        <v>39544</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="61">
       <c r="A24" s="9" t="inlineStr">
@@ -4135,6 +4450,9 @@
       <c r="F24" s="29" t="n">
         <v>10447</v>
       </c>
+      <c r="G24" s="29" t="n">
+        <v>8814</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="9" t="inlineStr">
@@ -4157,6 +4475,9 @@
       <c r="F25" s="29" t="n">
         <v>-7070</v>
       </c>
+      <c r="G25" s="29" t="n">
+        <v>-1799</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="12" t="inlineStr">
@@ -4179,6 +4500,9 @@
       <c r="F26" s="28" t="n">
         <v>-32211</v>
       </c>
+      <c r="G26" s="81" t="n">
+        <v>-5789</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="9" t="inlineStr">
@@ -4201,10 +4525,15 @@
       <c r="F27" s="29" t="n">
         <v>88538</v>
       </c>
+      <c r="G27" s="29">
+        <f>G23+G24+G25+G26</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -4214,15 +4543,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="61" min="1" max="1"/>
-    <col width="24" customWidth="1" style="61" min="2" max="2"/>
+    <col width="46" customWidth="1" style="61" min="1" max="1"/>
+    <col width="26" customWidth="1" style="61" min="2" max="2"/>
     <col width="13" customWidth="1" style="61" min="3" max="3"/>
-    <col width="13" customWidth="1" style="61" min="4" max="4"/>
-    <col width="13" customWidth="1" style="61" min="5" max="5"/>
-    <col width="42" customWidth="1" style="61" min="6" max="6"/>
+    <col width="10" customWidth="1" style="61" min="4" max="4"/>
+    <col width="16" customWidth="1" style="61" min="5" max="5"/>
+    <col width="62" customWidth="1" style="61" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4232,10 +4561,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>USD millions except per share. FY2025E segment basis. 12,200M shares; net cash ~$95bn. Live $370 (Jul 2026).</t>
+    <row r="2" ht="30" customHeight="1" s="61">
+      <c r="A2" s="84" t="inlineStr">
+        <is>
+          <t>USD millions except per share. Basis: Q2 2026A annualised run-rate. 12,360M fully diluted shares (incl. mandatory convertible preferred). Live $363.20 (5 Aug 2026, intraday).</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4583,7 @@
       </c>
       <c r="B6" s="72" t="inlineStr">
         <is>
-          <t>Metric (FY25E, $M)</t>
+          <t>Metric (Q2 2026A, $M)</t>
         </is>
       </c>
       <c r="C6" s="72" t="inlineStr">
@@ -4272,7 +4601,7 @@
           <t>EV / Value ($M)</t>
         </is>
       </c>
-      <c r="F6" s="72" t="inlineStr">
+      <c r="F6" s="85" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
@@ -4290,7 +4619,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>113000</v>
+        <v>113400</v>
       </c>
       <c r="D7" t="n">
         <v>25</v>
@@ -4299,9 +4628,9 @@
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Mature high-margin ads/subs @ 24x</t>
+      <c r="F7" s="84" t="inlineStr">
+        <is>
+          <t>Services op income $39.5bn/qtr less $5.8bn/qtr Alphabet-level AI R&amp;D, annualised, taxed at 16% → 25x</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4646,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>85000</v>
+        <v>99000</v>
       </c>
       <c r="D8" t="n">
         <v>21</v>
@@ -4326,9 +4655,9 @@
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Hyperscale @ 18x rev; +40-60% growth, $462bn RPO</t>
+      <c r="F8" s="84" t="inlineStr">
+        <is>
+          <t>Cloud Q2 revenue $24.8bn annualised (+82% YoY); $514bn backlog @ 21x revenue</t>
         </is>
       </c>
     </row>
@@ -4353,25 +4682,25 @@
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Waymo robotaxi lead + moonshots</t>
+      <c r="F9" s="84" t="inlineStr">
+        <is>
+          <t>Waymo robotaxi lead (Dallas now open-access) + moonshots</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Net cash</t>
+          <t>Net cash &amp; investments</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cash − debt</t>
+          <t>Cash+securities − debt + stakes</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>95000</v>
+        <v>246700</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -4380,9 +4709,9 @@
         <f>C10*D10</f>
         <v/>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Balance sheet</t>
+      <c r="F10" s="84" t="inlineStr">
+        <is>
+          <t>$242.5bn cash/securities − $98.2bn debt + $131.5bn non-marketable stakes net of 22% deferred tax</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4740,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12200</v>
+        <v>12360</v>
       </c>
     </row>
     <row r="15">
@@ -4432,7 +4761,7 @@
         </is>
       </c>
       <c r="B16" s="73" t="n">
-        <v>370</v>
+        <v>363.2</v>
       </c>
     </row>
     <row r="17">
@@ -4446,10 +4775,10 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Note: SOTP is the primary lens for a conglomerate — it surfaces Cloud value the blended-company P/E masks. Cross-checked against forward P/E (~30x FY26E EPS $13.7 → ~$410) and Street consensus (~$430). Blended fair value ~$400.</t>
+    <row r="19" ht="45" customHeight="1" s="61">
+      <c r="A19" s="84" t="inlineStr">
+        <is>
+          <t>Note: SOTP is the primary lens for a conglomerate — it surfaces Cloud value the blended-company P/E masks. Cross-checked against forward P/E on RECURRING earnings (30x FY26E EPS $11.90, which excludes the $135.7bn of H1-2026 unrealised equity gains) and Street consensus ($427.59). Blended fair value ~$384.</t>
         </is>
       </c>
     </row>
@@ -4474,21 +4803,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Forward P/E (35%): 30x × FY26E EPS $13.7</t>
+          <t>Forward P/E (35%): 30x × FY26E recurring EPS</t>
         </is>
       </c>
       <c r="B23" s="73" t="n">
-        <v>411</v>
+        <v>357</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DCF floor (20%)</t>
+          <t>DCF floor (20%) — cut for higher capex</t>
         </is>
       </c>
       <c r="B24" s="73" t="n">
-        <v>345</v>
+        <v>330</v>
       </c>
     </row>
     <row r="25">
@@ -4505,7 +4834,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Upside vs $370</t>
+          <t>Upside vs live price</t>
         </is>
       </c>
       <c r="B26" s="74">
@@ -4520,18 +4849,71 @@
         </is>
       </c>
       <c r="B27">
-        <f>IF(B26&gt;0.10,"BUY",IF(B26&gt;0.03,"ACCUMULATE",IF(B26&gt;-0.08,"HOLD","REDUCE")))</f>
-        <v/>
+        <f>IF(B29&gt;B30,"BUY",IF(B29&gt;B31,"ACCUMULATE",IF(B29&gt;0,"HOLD","REDUCE")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Dividend yield (FY26E DPS $0.88)</t>
+        </is>
+      </c>
+      <c r="B28" s="74">
+        <f>0.88/B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TOTAL RETURN (upside + dividend yield)</t>
+        </is>
+      </c>
+      <c r="B29" s="74">
+        <f>B26+B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BUY threshold — cost of equity (RF + 5.5% ERP)</t>
+        </is>
+      </c>
+      <c r="B30" s="74" t="n">
+        <v>0.1012</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ACCUMULATE threshold — RF + 2pp</t>
+        </is>
+      </c>
+      <c r="B31" s="74" t="n">
+        <v>0.06619999999999999</v>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1" s="61">
+      <c r="A33" s="84" t="inlineStr">
+        <is>
+          <t>Rating bands are anchored to the US 10-year Treasury (4.62%, 5 Aug 2026), not a fixed percentage: BUY if total return beats the ~10.1% cost of equity; ACCUMULATE above RF+2pp (6.6%); HOLD 0–6.6%; REDUCE below zero.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -4545,9 +4927,9 @@
   <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" style="61" min="1" max="1"/>
-    <col width="18" customWidth="1" style="61" min="2" max="2"/>
-    <col width="29.1640625" customWidth="1" style="61" min="3" max="3"/>
+    <col width="42" customWidth="1" style="61" min="1" max="1"/>
+    <col width="20" customWidth="1" style="61" min="2" max="2"/>
+    <col width="52" customWidth="1" style="61" min="3" max="3"/>
     <col width="12" customWidth="1" style="61" min="4" max="4"/>
     <col width="13" customWidth="1" style="61" min="5" max="5"/>
   </cols>
@@ -4559,14 +4941,14 @@
         </is>
       </c>
       <c r="B1" s="35" t="n"/>
-      <c r="C1" s="35" t="n"/>
+      <c r="C1" s="86" t="n"/>
       <c r="D1" s="36" t="n"/>
       <c r="E1" s="37" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="61">
       <c r="A2" s="5" t="n"/>
       <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
+      <c r="C2" s="87" t="n"/>
       <c r="D2" s="38" t="n"/>
       <c r="E2" s="38" t="n"/>
     </row>
@@ -4592,7 +4974,7 @@
           <t>Alphabet Inc. (Google)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n"/>
+      <c r="C4" s="87" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="61">
       <c r="A5" s="12" t="inlineStr">
@@ -4605,7 +4987,7 @@
           <t>GOOGL / GOOG</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n"/>
+      <c r="C5" s="89" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="61">
       <c r="A6" s="14" t="inlineStr">
@@ -4615,20 +4997,20 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>December 31, 2024</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n"/>
+          <t>December 31, 2025 (latest actual: Q2 2026)</t>
+        </is>
+      </c>
+      <c r="C6" s="87" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="87" t="n"/>
     </row>
     <row r="8" ht="18.75" customHeight="1" s="61">
       <c r="A8" s="69" t="inlineStr">
         <is>
-          <t>SECTION 2: CURRENT FINANCIAL DATA (FY 2024)</t>
+          <t>SECTION 2: LATEST FINANCIAL DATA (FY2025A; balance sheet &amp; shares at 30-Jun-2026)</t>
         </is>
       </c>
       <c r="B8" s="65" t="n"/>
@@ -4641,9 +5023,9 @@
         </is>
       </c>
       <c r="B9" s="30" t="n">
-        <v>350018</v>
-      </c>
-      <c r="C9" s="5" t="n"/>
+        <v>402836</v>
+      </c>
+      <c r="C9" s="87" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="61">
       <c r="A10" s="9" t="inlineStr">
@@ -4652,9 +5034,9 @@
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>88538</v>
-      </c>
-      <c r="C10" s="9" t="n"/>
+        <v>129039</v>
+      </c>
+      <c r="C10" s="90" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="61">
       <c r="A11" s="9" t="inlineStr">
@@ -4663,9 +5045,9 @@
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>82183</v>
-      </c>
-      <c r="C11" s="5" t="n"/>
+        <v>132170</v>
+      </c>
+      <c r="C11" s="87" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="61">
       <c r="A12" s="9" t="inlineStr">
@@ -4674,9 +5056,9 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>80769</v>
-      </c>
-      <c r="C12" s="9" t="n"/>
+        <v>73266</v>
+      </c>
+      <c r="C12" s="90" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="9" t="inlineStr">
@@ -4685,9 +5067,13 @@
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>16069</v>
-      </c>
-      <c r="C13" s="5" t="n"/>
+        <v>98165</v>
+      </c>
+      <c r="C13" s="91" t="inlineStr">
+        <is>
+          <t>← LT debt at 30-Jun-26</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="61">
       <c r="A14" s="12" t="inlineStr">
@@ -4696,9 +5082,13 @@
         </is>
       </c>
       <c r="B14" s="28" t="n">
-        <v>96635</v>
-      </c>
-      <c r="C14" s="12" t="n"/>
+        <v>242474</v>
+      </c>
+      <c r="C14" s="91" t="inlineStr">
+        <is>
+          <t>← cash + marketable securities, 30-Jun-26</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="61">
       <c r="A15" s="14" t="inlineStr">
@@ -4707,14 +5097,18 @@
         </is>
       </c>
       <c r="B15" s="30" t="n">
-        <v>10826</v>
-      </c>
-      <c r="C15" s="5" t="n"/>
+        <v>12309</v>
+      </c>
+      <c r="C15" s="91" t="inlineStr">
+        <is>
+          <t>← Q2 2026 diluted</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="61">
       <c r="A16" s="5" t="n"/>
       <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
+      <c r="C16" s="87" t="n"/>
     </row>
     <row r="17" ht="18.75" customHeight="1" s="61">
       <c r="A17" s="69" t="inlineStr">
@@ -4732,11 +5126,11 @@
         </is>
       </c>
       <c r="B18" s="41" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>← Adjust as needed</t>
+        <v>0.18</v>
+      </c>
+      <c r="C18" s="92" t="inlineStr">
+        <is>
+          <t>← FY26E consensus revenue growth +23.5%, tapering</t>
         </is>
       </c>
     </row>
@@ -4749,7 +5143,7 @@
       <c r="B19" s="24" t="n">
         <v>0.03</v>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="89" t="inlineStr">
         <is>
           <t>← Adjust as needed</t>
         </is>
@@ -4764,7 +5158,7 @@
       <c r="B20" s="41" t="n">
         <v>0.25</v>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="92" t="inlineStr">
         <is>
           <t>← Adjust as needed</t>
         </is>
@@ -4779,7 +5173,7 @@
       <c r="B21" s="24" t="n">
         <v>0.21</v>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="89" t="inlineStr">
         <is>
           <t>← Based on recent effective rate</t>
         </is>
@@ -4792,18 +5186,18 @@
         </is>
       </c>
       <c r="B22" s="41" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>← Adjust based on WACC calculation</t>
+        <v>0.09</v>
+      </c>
+      <c r="C22" s="92" t="inlineStr">
+        <is>
+          <t>← RF 4.62% + ERP 5.5% cost of equity, levered for $98bn debt</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="61">
       <c r="A23" s="5" t="n"/>
       <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
+      <c r="C23" s="87" t="n"/>
     </row>
     <row r="24" ht="18.75" customHeight="1" s="61">
       <c r="A24" s="69" t="inlineStr">
@@ -4821,53 +5215,53 @@
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>370.21</v>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>← live 16 Jul 2026</t>
+        <v>363.2</v>
+      </c>
+      <c r="C25" s="92" t="inlineStr">
+        <is>
+          <t>← live 5 Aug 2026 (intraday)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Diluted EPS (FY 2024)</t>
+          <t>Diluted EPS (FY2025A)</t>
         </is>
       </c>
       <c r="B26" s="42" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="C26" s="12" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="61">
+        <v>10.81</v>
+      </c>
+      <c r="C26" s="89" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1" s="61">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>Forward EPS (FY 2025E)</t>
+          <t>Forward EPS (FY2026E, recurring)</t>
         </is>
       </c>
       <c r="B27" s="14" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>← FY2026E consensus</t>
+        <v>11.9</v>
+      </c>
+      <c r="C27" s="92" t="inlineStr">
+        <is>
+          <t>← ex unrealised equity gains (GAAP consensus $20.58 is inflated by them)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="61">
       <c r="A28" s="5" t="n"/>
       <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
+      <c r="C28" s="87" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>SECTION 5: COMPARABLE COMPANIES</t>
+          <t>SECTION 5: COMPARABLE COMPANIES (live 5 Aug 2026)</t>
         </is>
       </c>
       <c r="B29" s="26" t="n"/>
-      <c r="C29" s="26" t="n"/>
+      <c r="C29" s="93" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="61">
       <c r="A30" s="14" t="inlineStr">
@@ -4880,7 +5274,7 @@
           <t>PE Ratio</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="92" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
@@ -4892,15 +5286,11 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
+      <c r="B31" s="12" t="n">
+        <v>27.45</v>
+      </c>
+      <c r="C31" s="89" t="n">
+        <v>3640000</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="61">
@@ -4909,15 +5299,11 @@
           <t>Apple</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
+      <c r="B32" s="14" t="n">
+        <v>35.49</v>
+      </c>
+      <c r="C32" s="92" t="n">
+        <v>4500000</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="61">
@@ -4926,15 +5312,11 @@
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
+      <c r="B33" s="12" t="n">
+        <v>22.15</v>
+      </c>
+      <c r="C33" s="89" t="n">
+        <v>1490000</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="61">
@@ -4943,15 +5325,11 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t>Enter</t>
-        </is>
+      <c r="B34" s="14" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="C34" s="92" t="n">
+        <v>2930000</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="61">
@@ -4960,17 +5338,16 @@
           <t>Industry Average PE</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>Calculate</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="n"/>
+      <c r="B35" s="12">
+        <f>MEDIAN(B31:B34)</f>
+        <v/>
+      </c>
+      <c r="C35" s="89" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="61">
       <c r="A36" s="5" t="n"/>
       <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
+      <c r="C36" s="87" t="n"/>
     </row>
     <row r="37" ht="18.75" customHeight="1" s="61">
       <c r="A37" s="69" t="inlineStr">
@@ -4988,7 +5365,7 @@
         </is>
       </c>
       <c r="B38" s="26" t="n"/>
-      <c r="C38" s="26" t="n"/>
+      <c r="C38" s="93" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="61">
       <c r="A39" s="16" t="inlineStr">
@@ -4997,7 +5374,7 @@
         </is>
       </c>
       <c r="B39" s="26" t="n"/>
-      <c r="C39" s="26" t="n"/>
+      <c r="C39" s="93" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="61">
       <c r="A40" s="16" t="inlineStr">
@@ -5006,7 +5383,7 @@
         </is>
       </c>
       <c r="B40" s="26" t="n"/>
-      <c r="C40" s="26" t="n"/>
+      <c r="C40" s="93" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="61">
       <c r="A41" s="16" t="inlineStr">
@@ -5015,7 +5392,7 @@
         </is>
       </c>
       <c r="B41" s="26" t="n"/>
-      <c r="C41" s="26" t="n"/>
+      <c r="C41" s="93" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="61">
       <c r="A42" s="16" t="inlineStr">
@@ -5024,7 +5401,7 @@
         </is>
       </c>
       <c r="B42" s="26" t="n"/>
-      <c r="C42" s="26" t="n"/>
+      <c r="C42" s="93" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="61">
       <c r="A43" s="16" t="inlineStr">
@@ -5033,7 +5410,7 @@
         </is>
       </c>
       <c r="B43" s="26" t="n"/>
-      <c r="C43" s="26" t="n"/>
+      <c r="C43" s="93" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5043,8 +5420,9 @@
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A24:C24"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -5058,8 +5436,10 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" style="61" min="1" max="1"/>
+    <col width="42" customWidth="1" style="61" min="1" max="1"/>
     <col width="14" customWidth="1" style="61" min="2" max="4"/>
+    <col width="14" customWidth="1" style="61" min="3" max="3"/>
+    <col width="14" customWidth="1" style="61" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="61">
@@ -5072,7 +5452,7 @@
     <row r="2">
       <c r="A2" s="63" t="inlineStr">
         <is>
-          <t>Researched Jul 2026 · live prices as of 15-16 Jul 2026</t>
+          <t>Researched Aug 2026 · live prices as of 5 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -5105,10 +5485,10 @@
         </is>
       </c>
       <c r="B5" s="46" t="n">
-        <v>370.21</v>
+        <v>363.2</v>
       </c>
       <c r="C5" s="46" t="n">
-        <v>13.24</v>
+        <v>11.9</v>
       </c>
       <c r="D5" s="47">
         <f>B5/C5</f>
@@ -5122,10 +5502,10 @@
         </is>
       </c>
       <c r="B6" s="49" t="n">
-        <v>281.74</v>
+        <v>308.57</v>
       </c>
       <c r="C6" s="49" t="n">
-        <v>8.289999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="D6" s="50">
         <f>B6/C6</f>
@@ -5139,10 +5519,10 @@
         </is>
       </c>
       <c r="B7" s="52" t="n">
-        <v>395.63</v>
+        <v>490</v>
       </c>
       <c r="C7" s="52" t="n">
-        <v>16.86</v>
+        <v>17.85</v>
       </c>
       <c r="D7" s="53">
         <f>B7/C7</f>
@@ -5156,10 +5536,10 @@
         </is>
       </c>
       <c r="B8" s="49" t="n">
-        <v>254.96</v>
+        <v>271.77</v>
       </c>
       <c r="C8" s="49" t="n">
-        <v>8.49</v>
+        <v>12.18</v>
       </c>
       <c r="D8" s="50">
         <f>B8/C8</f>
@@ -5173,10 +5553,10 @@
         </is>
       </c>
       <c r="B9" s="52" t="n">
-        <v>679.9400000000001</v>
+        <v>583.48</v>
       </c>
       <c r="C9" s="52" t="n">
-        <v>27.95</v>
+        <v>26.34</v>
       </c>
       <c r="D9" s="53">
         <f>B9/C9</f>
@@ -5237,10 +5617,10 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="72" customHeight="1" s="61">
       <c r="A17" s="62" t="inlineStr">
         <is>
-          <t>Note: Alphabet sits mid-pack on trailing P/E despite the strongest cloud/AI growth in the group — the basis of the BUY: quality growth at a market multiple.</t>
+          <t>Note: Alphabet is shown on FY2026E RECURRING EPS ($11.90, ex the $135.7bn of H1-2026 unrealised equity gains); peers are on trailing EPS. The headline 18.9x trailing P/E screens cheap only because those gains inflate GAAP earnings — on recurring earnings Alphabet trades at a premium to the mega-cap median, which is why the comps cross-check now sits below the current price rather than above it.</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5633,8 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D11"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>